<commit_message>
test(core): add cell borders to table-each fixture and assert they survive jx:each
The table-each template now applies thin borders to all 9 cells of the
3x3 layout (header, template data row, totals row). EndToEndTest verifies
that JXLS copies the border style onto every generated row when the
template row is duplicated by jx:each, so the totals row stays bordered
after it is pushed down past the expanded items.

SampleTemplateGenerator is split into per-fixture methods so a single
template can be regenerated when others are open in Excel.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc-engine-core/src/test/resources/templates/table-each.xlsx
+++ b/doc-engine-core/src/test/resources/templates/table-each.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Name</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>${item.qty * item.price}</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -74,7 +77,7 @@
       <patternFill patternType="darkGray"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -82,12 +85,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -102,32 +124,35 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="1">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="1">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="1">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="B3" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1">
         <f>SUM(C2:C2)</f>
       </c>
     </row>

</xml_diff>